<commit_message>
Added placeholder for cart# and bag#
</commit_message>
<xml_diff>
--- a/templates/excel/MatchAid_GameTeeSheet_Template.xlsx
+++ b/templates/excel/MatchAid_GameTeeSheet_Template.xlsx
@@ -14,8 +14,8 @@
   <definedNames>
     <definedName name="Hdr_Title" localSheetId="0">'By Playing Group'!$A$1</definedName>
     <definedName name="Hdr_SubLine" localSheetId="0">'By Playing Group'!$A$2</definedName>
-    <definedName name="GroupBand" localSheetId="0">'By Playing Group'!$A$5:$I$8</definedName>
-    <definedName name="GroupBands" localSheetId="0">'By Playing Group'!$A$5:$I$84</definedName>
+    <definedName name="GroupBand" localSheetId="0">'By Playing Group'!$A$5:$K$8</definedName>
+    <definedName name="GroupBands" localSheetId="0">'By Playing Group'!$A$5:$K$84</definedName>
     <definedName name="Band_L_Time" localSheetId="0">'By Playing Group'!$A$5</definedName>
     <definedName name="Band_L_Hole" localSheetId="0">'By Playing Group'!$B$5</definedName>
     <definedName name="Band_L_Player1" localSheetId="0">'By Playing Group'!$C$5</definedName>
@@ -28,20 +28,22 @@
     <definedName name="Band_L_Cart4" localSheetId="0">'By Playing Group'!$D$8</definedName>
     <definedName name="Col_L_Time" localSheetId="0">'By Playing Group'!$A$4:$A$84</definedName>
     <definedName name="Col_L_Cart" localSheetId="0">'By Playing Group'!$D$4:$D$84</definedName>
-    <definedName name="Band_R_Time" localSheetId="0">'By Playing Group'!$F$5</definedName>
-    <definedName name="Band_R_Hole" localSheetId="0">'By Playing Group'!$G$5</definedName>
-    <definedName name="Band_R_Player1" localSheetId="0">'By Playing Group'!$H$5</definedName>
-    <definedName name="Band_R_Cart1" localSheetId="0">'By Playing Group'!$I$5</definedName>
-    <definedName name="Band_R_Player2" localSheetId="0">'By Playing Group'!$H$6</definedName>
-    <definedName name="Band_R_Cart2" localSheetId="0">'By Playing Group'!$I$6</definedName>
-    <definedName name="Band_R_Player3" localSheetId="0">'By Playing Group'!$H$7</definedName>
-    <definedName name="Band_R_Cart3" localSheetId="0">'By Playing Group'!$I$7</definedName>
-    <definedName name="Band_R_Player4" localSheetId="0">'By Playing Group'!$H$8</definedName>
-    <definedName name="Band_R_Cart4" localSheetId="0">'By Playing Group'!$I$8</definedName>
-    <definedName name="Col_R_Time" localSheetId="0">'By Playing Group'!$F$4:$F$84</definedName>
-    <definedName name="Col_R_Cart" localSheetId="0">'By Playing Group'!$I$4:$I$84</definedName>
+    <definedName name="Col_L_Bag" localSheetId="0">'By Playing Group'!$E$4:$E$84</definedName>
+    <definedName name="Band_R_Time" localSheetId="0">'By Playing Group'!$G$5</definedName>
+    <definedName name="Band_R_Hole" localSheetId="0">'By Playing Group'!$H$5</definedName>
+    <definedName name="Band_R_Player1" localSheetId="0">'By Playing Group'!$I$5</definedName>
+    <definedName name="Band_R_Cart1" localSheetId="0">'By Playing Group'!$J$5</definedName>
+    <definedName name="Band_R_Player2" localSheetId="0">'By Playing Group'!$I$6</definedName>
+    <definedName name="Band_R_Cart2" localSheetId="0">'By Playing Group'!$J$6</definedName>
+    <definedName name="Band_R_Player3" localSheetId="0">'By Playing Group'!$I$7</definedName>
+    <definedName name="Band_R_Cart3" localSheetId="0">'By Playing Group'!$J$7</definedName>
+    <definedName name="Band_R_Player4" localSheetId="0">'By Playing Group'!$I$8</definedName>
+    <definedName name="Band_R_Cart4" localSheetId="0">'By Playing Group'!$J$8</definedName>
+    <definedName name="Col_R_Time" localSheetId="0">'By Playing Group'!$G$4:$G$84</definedName>
+    <definedName name="Col_R_Cart" localSheetId="0">'By Playing Group'!$J$4:$J$84</definedName>
+    <definedName name="Col_R_Bag" localSheetId="0">'By Playing Group'!$K$4:$K$84</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'By Playing Group'!$1:$4</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'By Playing Group'!$A$1:$I$84</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'By Playing Group'!$A$1:$K$84</definedName>
     <definedName name="Hdr_Title" localSheetId="1">'By Individual'!$A$1</definedName>
     <definedName name="Hdr_SubLine" localSheetId="1">'By Individual'!$A$2</definedName>
     <definedName name="DetailRow" localSheetId="1">'By Individual'!$A$5:$G$5</definedName>
@@ -710,18 +712,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I84"/>
+  <dimension ref="A1:K84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="6" customWidth="1" min="4" max="4"/>
-    <col width="2" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="6" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="6" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="2" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="6" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -757,27 +761,37 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Cart</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
+          <t>Cart #</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Bag #</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Hole</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Players</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>Cart</t>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Cart #</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>Bag #</t>
         </is>
       </c>
     </row>
@@ -785,806 +799,966 @@
       <c r="A5" s="5" t="n"/>
       <c r="B5" s="6" t="n"/>
       <c r="C5" s="7" t="n"/>
-      <c r="D5" s="8" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="7" t="n"/>
-      <c r="I5" s="8" t="n"/>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="8" t="n"/>
+      <c r="G5" s="5" t="n"/>
+      <c r="H5" s="6" t="n"/>
+      <c r="I5" s="7" t="n"/>
+      <c r="J5" s="6" t="n"/>
+      <c r="K5" s="8" t="n"/>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="9" t="n"/>
       <c r="B6" s="10" t="n"/>
       <c r="C6" s="11" t="n"/>
-      <c r="D6" s="12" t="n"/>
-      <c r="F6" s="9" t="n"/>
-      <c r="G6" s="10" t="n"/>
-      <c r="H6" s="11" t="n"/>
-      <c r="I6" s="12" t="n"/>
+      <c r="D6" s="10" t="n"/>
+      <c r="E6" s="12" t="n"/>
+      <c r="G6" s="9" t="n"/>
+      <c r="H6" s="10" t="n"/>
+      <c r="I6" s="11" t="n"/>
+      <c r="J6" s="10" t="n"/>
+      <c r="K6" s="12" t="n"/>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="9" t="n"/>
       <c r="B7" s="10" t="n"/>
       <c r="C7" s="11" t="n"/>
-      <c r="D7" s="12" t="n"/>
-      <c r="F7" s="9" t="n"/>
-      <c r="G7" s="10" t="n"/>
-      <c r="H7" s="11" t="n"/>
-      <c r="I7" s="12" t="n"/>
+      <c r="D7" s="10" t="n"/>
+      <c r="E7" s="12" t="n"/>
+      <c r="G7" s="9" t="n"/>
+      <c r="H7" s="10" t="n"/>
+      <c r="I7" s="11" t="n"/>
+      <c r="J7" s="10" t="n"/>
+      <c r="K7" s="12" t="n"/>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="13" t="n"/>
       <c r="B8" s="14" t="n"/>
       <c r="C8" s="15" t="n"/>
-      <c r="D8" s="16" t="n"/>
-      <c r="F8" s="13" t="n"/>
-      <c r="G8" s="14" t="n"/>
-      <c r="H8" s="15" t="n"/>
-      <c r="I8" s="16" t="n"/>
+      <c r="D8" s="14" t="n"/>
+      <c r="E8" s="16" t="n"/>
+      <c r="G8" s="13" t="n"/>
+      <c r="H8" s="14" t="n"/>
+      <c r="I8" s="15" t="n"/>
+      <c r="J8" s="14" t="n"/>
+      <c r="K8" s="16" t="n"/>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="17" t="n"/>
       <c r="B9" s="18" t="n"/>
       <c r="C9" s="19" t="n"/>
-      <c r="D9" s="20" t="n"/>
-      <c r="F9" s="17" t="n"/>
-      <c r="G9" s="18" t="n"/>
-      <c r="H9" s="19" t="n"/>
-      <c r="I9" s="20" t="n"/>
+      <c r="D9" s="18" t="n"/>
+      <c r="E9" s="20" t="n"/>
+      <c r="G9" s="17" t="n"/>
+      <c r="H9" s="18" t="n"/>
+      <c r="I9" s="19" t="n"/>
+      <c r="J9" s="18" t="n"/>
+      <c r="K9" s="20" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="21" t="n"/>
       <c r="B10" s="22" t="n"/>
       <c r="C10" s="23" t="n"/>
-      <c r="D10" s="24" t="n"/>
-      <c r="F10" s="21" t="n"/>
-      <c r="G10" s="22" t="n"/>
-      <c r="H10" s="23" t="n"/>
-      <c r="I10" s="24" t="n"/>
+      <c r="D10" s="22" t="n"/>
+      <c r="E10" s="24" t="n"/>
+      <c r="G10" s="21" t="n"/>
+      <c r="H10" s="22" t="n"/>
+      <c r="I10" s="23" t="n"/>
+      <c r="J10" s="22" t="n"/>
+      <c r="K10" s="24" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="21" t="n"/>
       <c r="B11" s="22" t="n"/>
       <c r="C11" s="23" t="n"/>
-      <c r="D11" s="24" t="n"/>
-      <c r="F11" s="21" t="n"/>
-      <c r="G11" s="22" t="n"/>
-      <c r="H11" s="23" t="n"/>
-      <c r="I11" s="24" t="n"/>
+      <c r="D11" s="22" t="n"/>
+      <c r="E11" s="24" t="n"/>
+      <c r="G11" s="21" t="n"/>
+      <c r="H11" s="22" t="n"/>
+      <c r="I11" s="23" t="n"/>
+      <c r="J11" s="22" t="n"/>
+      <c r="K11" s="24" t="n"/>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="25" t="n"/>
       <c r="B12" s="26" t="n"/>
       <c r="C12" s="27" t="n"/>
-      <c r="D12" s="28" t="n"/>
-      <c r="F12" s="25" t="n"/>
-      <c r="G12" s="26" t="n"/>
-      <c r="H12" s="27" t="n"/>
-      <c r="I12" s="28" t="n"/>
+      <c r="D12" s="26" t="n"/>
+      <c r="E12" s="28" t="n"/>
+      <c r="G12" s="25" t="n"/>
+      <c r="H12" s="26" t="n"/>
+      <c r="I12" s="27" t="n"/>
+      <c r="J12" s="26" t="n"/>
+      <c r="K12" s="28" t="n"/>
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="5" t="n"/>
       <c r="B13" s="6" t="n"/>
       <c r="C13" s="7" t="n"/>
-      <c r="D13" s="8" t="n"/>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="6" t="n"/>
-      <c r="H13" s="7" t="n"/>
-      <c r="I13" s="8" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="8" t="n"/>
+      <c r="G13" s="5" t="n"/>
+      <c r="H13" s="6" t="n"/>
+      <c r="I13" s="7" t="n"/>
+      <c r="J13" s="6" t="n"/>
+      <c r="K13" s="8" t="n"/>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="9" t="n"/>
       <c r="B14" s="10" t="n"/>
       <c r="C14" s="11" t="n"/>
-      <c r="D14" s="12" t="n"/>
-      <c r="F14" s="9" t="n"/>
-      <c r="G14" s="10" t="n"/>
-      <c r="H14" s="11" t="n"/>
-      <c r="I14" s="12" t="n"/>
+      <c r="D14" s="10" t="n"/>
+      <c r="E14" s="12" t="n"/>
+      <c r="G14" s="9" t="n"/>
+      <c r="H14" s="10" t="n"/>
+      <c r="I14" s="11" t="n"/>
+      <c r="J14" s="10" t="n"/>
+      <c r="K14" s="12" t="n"/>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="9" t="n"/>
       <c r="B15" s="10" t="n"/>
       <c r="C15" s="11" t="n"/>
-      <c r="D15" s="12" t="n"/>
-      <c r="F15" s="9" t="n"/>
-      <c r="G15" s="10" t="n"/>
-      <c r="H15" s="11" t="n"/>
-      <c r="I15" s="12" t="n"/>
+      <c r="D15" s="10" t="n"/>
+      <c r="E15" s="12" t="n"/>
+      <c r="G15" s="9" t="n"/>
+      <c r="H15" s="10" t="n"/>
+      <c r="I15" s="11" t="n"/>
+      <c r="J15" s="10" t="n"/>
+      <c r="K15" s="12" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="13" t="n"/>
       <c r="B16" s="14" t="n"/>
       <c r="C16" s="15" t="n"/>
-      <c r="D16" s="16" t="n"/>
-      <c r="F16" s="13" t="n"/>
-      <c r="G16" s="14" t="n"/>
-      <c r="H16" s="15" t="n"/>
-      <c r="I16" s="16" t="n"/>
+      <c r="D16" s="14" t="n"/>
+      <c r="E16" s="16" t="n"/>
+      <c r="G16" s="13" t="n"/>
+      <c r="H16" s="14" t="n"/>
+      <c r="I16" s="15" t="n"/>
+      <c r="J16" s="14" t="n"/>
+      <c r="K16" s="16" t="n"/>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="17" t="n"/>
       <c r="B17" s="18" t="n"/>
       <c r="C17" s="19" t="n"/>
-      <c r="D17" s="20" t="n"/>
-      <c r="F17" s="17" t="n"/>
-      <c r="G17" s="18" t="n"/>
-      <c r="H17" s="19" t="n"/>
-      <c r="I17" s="20" t="n"/>
+      <c r="D17" s="18" t="n"/>
+      <c r="E17" s="20" t="n"/>
+      <c r="G17" s="17" t="n"/>
+      <c r="H17" s="18" t="n"/>
+      <c r="I17" s="19" t="n"/>
+      <c r="J17" s="18" t="n"/>
+      <c r="K17" s="20" t="n"/>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="21" t="n"/>
       <c r="B18" s="22" t="n"/>
       <c r="C18" s="23" t="n"/>
-      <c r="D18" s="24" t="n"/>
-      <c r="F18" s="21" t="n"/>
-      <c r="G18" s="22" t="n"/>
-      <c r="H18" s="23" t="n"/>
-      <c r="I18" s="24" t="n"/>
+      <c r="D18" s="22" t="n"/>
+      <c r="E18" s="24" t="n"/>
+      <c r="G18" s="21" t="n"/>
+      <c r="H18" s="22" t="n"/>
+      <c r="I18" s="23" t="n"/>
+      <c r="J18" s="22" t="n"/>
+      <c r="K18" s="24" t="n"/>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="21" t="n"/>
       <c r="B19" s="22" t="n"/>
       <c r="C19" s="23" t="n"/>
-      <c r="D19" s="24" t="n"/>
-      <c r="F19" s="21" t="n"/>
-      <c r="G19" s="22" t="n"/>
-      <c r="H19" s="23" t="n"/>
-      <c r="I19" s="24" t="n"/>
+      <c r="D19" s="22" t="n"/>
+      <c r="E19" s="24" t="n"/>
+      <c r="G19" s="21" t="n"/>
+      <c r="H19" s="22" t="n"/>
+      <c r="I19" s="23" t="n"/>
+      <c r="J19" s="22" t="n"/>
+      <c r="K19" s="24" t="n"/>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="25" t="n"/>
       <c r="B20" s="26" t="n"/>
       <c r="C20" s="27" t="n"/>
-      <c r="D20" s="28" t="n"/>
-      <c r="F20" s="25" t="n"/>
-      <c r="G20" s="26" t="n"/>
-      <c r="H20" s="27" t="n"/>
-      <c r="I20" s="28" t="n"/>
+      <c r="D20" s="26" t="n"/>
+      <c r="E20" s="28" t="n"/>
+      <c r="G20" s="25" t="n"/>
+      <c r="H20" s="26" t="n"/>
+      <c r="I20" s="27" t="n"/>
+      <c r="J20" s="26" t="n"/>
+      <c r="K20" s="28" t="n"/>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="5" t="n"/>
       <c r="B21" s="6" t="n"/>
       <c r="C21" s="7" t="n"/>
-      <c r="D21" s="8" t="n"/>
-      <c r="F21" s="5" t="n"/>
-      <c r="G21" s="6" t="n"/>
-      <c r="H21" s="7" t="n"/>
-      <c r="I21" s="8" t="n"/>
+      <c r="D21" s="6" t="n"/>
+      <c r="E21" s="8" t="n"/>
+      <c r="G21" s="5" t="n"/>
+      <c r="H21" s="6" t="n"/>
+      <c r="I21" s="7" t="n"/>
+      <c r="J21" s="6" t="n"/>
+      <c r="K21" s="8" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="9" t="n"/>
       <c r="B22" s="10" t="n"/>
       <c r="C22" s="11" t="n"/>
-      <c r="D22" s="12" t="n"/>
-      <c r="F22" s="9" t="n"/>
-      <c r="G22" s="10" t="n"/>
-      <c r="H22" s="11" t="n"/>
-      <c r="I22" s="12" t="n"/>
+      <c r="D22" s="10" t="n"/>
+      <c r="E22" s="12" t="n"/>
+      <c r="G22" s="9" t="n"/>
+      <c r="H22" s="10" t="n"/>
+      <c r="I22" s="11" t="n"/>
+      <c r="J22" s="10" t="n"/>
+      <c r="K22" s="12" t="n"/>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="9" t="n"/>
       <c r="B23" s="10" t="n"/>
       <c r="C23" s="11" t="n"/>
-      <c r="D23" s="12" t="n"/>
-      <c r="F23" s="9" t="n"/>
-      <c r="G23" s="10" t="n"/>
-      <c r="H23" s="11" t="n"/>
-      <c r="I23" s="12" t="n"/>
+      <c r="D23" s="10" t="n"/>
+      <c r="E23" s="12" t="n"/>
+      <c r="G23" s="9" t="n"/>
+      <c r="H23" s="10" t="n"/>
+      <c r="I23" s="11" t="n"/>
+      <c r="J23" s="10" t="n"/>
+      <c r="K23" s="12" t="n"/>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="13" t="n"/>
       <c r="B24" s="14" t="n"/>
       <c r="C24" s="15" t="n"/>
-      <c r="D24" s="16" t="n"/>
-      <c r="F24" s="13" t="n"/>
-      <c r="G24" s="14" t="n"/>
-      <c r="H24" s="15" t="n"/>
-      <c r="I24" s="16" t="n"/>
+      <c r="D24" s="14" t="n"/>
+      <c r="E24" s="16" t="n"/>
+      <c r="G24" s="13" t="n"/>
+      <c r="H24" s="14" t="n"/>
+      <c r="I24" s="15" t="n"/>
+      <c r="J24" s="14" t="n"/>
+      <c r="K24" s="16" t="n"/>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="17" t="n"/>
       <c r="B25" s="18" t="n"/>
       <c r="C25" s="19" t="n"/>
-      <c r="D25" s="20" t="n"/>
-      <c r="F25" s="17" t="n"/>
-      <c r="G25" s="18" t="n"/>
-      <c r="H25" s="19" t="n"/>
-      <c r="I25" s="20" t="n"/>
+      <c r="D25" s="18" t="n"/>
+      <c r="E25" s="20" t="n"/>
+      <c r="G25" s="17" t="n"/>
+      <c r="H25" s="18" t="n"/>
+      <c r="I25" s="19" t="n"/>
+      <c r="J25" s="18" t="n"/>
+      <c r="K25" s="20" t="n"/>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="21" t="n"/>
       <c r="B26" s="22" t="n"/>
       <c r="C26" s="23" t="n"/>
-      <c r="D26" s="24" t="n"/>
-      <c r="F26" s="21" t="n"/>
-      <c r="G26" s="22" t="n"/>
-      <c r="H26" s="23" t="n"/>
-      <c r="I26" s="24" t="n"/>
+      <c r="D26" s="22" t="n"/>
+      <c r="E26" s="24" t="n"/>
+      <c r="G26" s="21" t="n"/>
+      <c r="H26" s="22" t="n"/>
+      <c r="I26" s="23" t="n"/>
+      <c r="J26" s="22" t="n"/>
+      <c r="K26" s="24" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="21" t="n"/>
       <c r="B27" s="22" t="n"/>
       <c r="C27" s="23" t="n"/>
-      <c r="D27" s="24" t="n"/>
-      <c r="F27" s="21" t="n"/>
-      <c r="G27" s="22" t="n"/>
-      <c r="H27" s="23" t="n"/>
-      <c r="I27" s="24" t="n"/>
+      <c r="D27" s="22" t="n"/>
+      <c r="E27" s="24" t="n"/>
+      <c r="G27" s="21" t="n"/>
+      <c r="H27" s="22" t="n"/>
+      <c r="I27" s="23" t="n"/>
+      <c r="J27" s="22" t="n"/>
+      <c r="K27" s="24" t="n"/>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="25" t="n"/>
       <c r="B28" s="26" t="n"/>
       <c r="C28" s="27" t="n"/>
-      <c r="D28" s="28" t="n"/>
-      <c r="F28" s="25" t="n"/>
-      <c r="G28" s="26" t="n"/>
-      <c r="H28" s="27" t="n"/>
-      <c r="I28" s="28" t="n"/>
+      <c r="D28" s="26" t="n"/>
+      <c r="E28" s="28" t="n"/>
+      <c r="G28" s="25" t="n"/>
+      <c r="H28" s="26" t="n"/>
+      <c r="I28" s="27" t="n"/>
+      <c r="J28" s="26" t="n"/>
+      <c r="K28" s="28" t="n"/>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="5" t="n"/>
       <c r="B29" s="6" t="n"/>
       <c r="C29" s="7" t="n"/>
-      <c r="D29" s="8" t="n"/>
-      <c r="F29" s="5" t="n"/>
-      <c r="G29" s="6" t="n"/>
-      <c r="H29" s="7" t="n"/>
-      <c r="I29" s="8" t="n"/>
+      <c r="D29" s="6" t="n"/>
+      <c r="E29" s="8" t="n"/>
+      <c r="G29" s="5" t="n"/>
+      <c r="H29" s="6" t="n"/>
+      <c r="I29" s="7" t="n"/>
+      <c r="J29" s="6" t="n"/>
+      <c r="K29" s="8" t="n"/>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="9" t="n"/>
       <c r="B30" s="10" t="n"/>
       <c r="C30" s="11" t="n"/>
-      <c r="D30" s="12" t="n"/>
-      <c r="F30" s="9" t="n"/>
-      <c r="G30" s="10" t="n"/>
-      <c r="H30" s="11" t="n"/>
-      <c r="I30" s="12" t="n"/>
+      <c r="D30" s="10" t="n"/>
+      <c r="E30" s="12" t="n"/>
+      <c r="G30" s="9" t="n"/>
+      <c r="H30" s="10" t="n"/>
+      <c r="I30" s="11" t="n"/>
+      <c r="J30" s="10" t="n"/>
+      <c r="K30" s="12" t="n"/>
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="9" t="n"/>
       <c r="B31" s="10" t="n"/>
       <c r="C31" s="11" t="n"/>
-      <c r="D31" s="12" t="n"/>
-      <c r="F31" s="9" t="n"/>
-      <c r="G31" s="10" t="n"/>
-      <c r="H31" s="11" t="n"/>
-      <c r="I31" s="12" t="n"/>
+      <c r="D31" s="10" t="n"/>
+      <c r="E31" s="12" t="n"/>
+      <c r="G31" s="9" t="n"/>
+      <c r="H31" s="10" t="n"/>
+      <c r="I31" s="11" t="n"/>
+      <c r="J31" s="10" t="n"/>
+      <c r="K31" s="12" t="n"/>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="13" t="n"/>
       <c r="B32" s="14" t="n"/>
       <c r="C32" s="15" t="n"/>
-      <c r="D32" s="16" t="n"/>
-      <c r="F32" s="13" t="n"/>
-      <c r="G32" s="14" t="n"/>
-      <c r="H32" s="15" t="n"/>
-      <c r="I32" s="16" t="n"/>
+      <c r="D32" s="14" t="n"/>
+      <c r="E32" s="16" t="n"/>
+      <c r="G32" s="13" t="n"/>
+      <c r="H32" s="14" t="n"/>
+      <c r="I32" s="15" t="n"/>
+      <c r="J32" s="14" t="n"/>
+      <c r="K32" s="16" t="n"/>
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="A33" s="17" t="n"/>
       <c r="B33" s="18" t="n"/>
       <c r="C33" s="19" t="n"/>
-      <c r="D33" s="20" t="n"/>
-      <c r="F33" s="17" t="n"/>
-      <c r="G33" s="18" t="n"/>
-      <c r="H33" s="19" t="n"/>
-      <c r="I33" s="20" t="n"/>
+      <c r="D33" s="18" t="n"/>
+      <c r="E33" s="20" t="n"/>
+      <c r="G33" s="17" t="n"/>
+      <c r="H33" s="18" t="n"/>
+      <c r="I33" s="19" t="n"/>
+      <c r="J33" s="18" t="n"/>
+      <c r="K33" s="20" t="n"/>
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="A34" s="21" t="n"/>
       <c r="B34" s="22" t="n"/>
       <c r="C34" s="23" t="n"/>
-      <c r="D34" s="24" t="n"/>
-      <c r="F34" s="21" t="n"/>
-      <c r="G34" s="22" t="n"/>
-      <c r="H34" s="23" t="n"/>
-      <c r="I34" s="24" t="n"/>
+      <c r="D34" s="22" t="n"/>
+      <c r="E34" s="24" t="n"/>
+      <c r="G34" s="21" t="n"/>
+      <c r="H34" s="22" t="n"/>
+      <c r="I34" s="23" t="n"/>
+      <c r="J34" s="22" t="n"/>
+      <c r="K34" s="24" t="n"/>
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="A35" s="21" t="n"/>
       <c r="B35" s="22" t="n"/>
       <c r="C35" s="23" t="n"/>
-      <c r="D35" s="24" t="n"/>
-      <c r="F35" s="21" t="n"/>
-      <c r="G35" s="22" t="n"/>
-      <c r="H35" s="23" t="n"/>
-      <c r="I35" s="24" t="n"/>
+      <c r="D35" s="22" t="n"/>
+      <c r="E35" s="24" t="n"/>
+      <c r="G35" s="21" t="n"/>
+      <c r="H35" s="22" t="n"/>
+      <c r="I35" s="23" t="n"/>
+      <c r="J35" s="22" t="n"/>
+      <c r="K35" s="24" t="n"/>
     </row>
     <row r="36" ht="15" customHeight="1">
       <c r="A36" s="25" t="n"/>
       <c r="B36" s="26" t="n"/>
       <c r="C36" s="27" t="n"/>
-      <c r="D36" s="28" t="n"/>
-      <c r="F36" s="25" t="n"/>
-      <c r="G36" s="26" t="n"/>
-      <c r="H36" s="27" t="n"/>
-      <c r="I36" s="28" t="n"/>
+      <c r="D36" s="26" t="n"/>
+      <c r="E36" s="28" t="n"/>
+      <c r="G36" s="25" t="n"/>
+      <c r="H36" s="26" t="n"/>
+      <c r="I36" s="27" t="n"/>
+      <c r="J36" s="26" t="n"/>
+      <c r="K36" s="28" t="n"/>
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="A37" s="5" t="n"/>
       <c r="B37" s="6" t="n"/>
       <c r="C37" s="7" t="n"/>
-      <c r="D37" s="8" t="n"/>
-      <c r="F37" s="5" t="n"/>
-      <c r="G37" s="6" t="n"/>
-      <c r="H37" s="7" t="n"/>
-      <c r="I37" s="8" t="n"/>
+      <c r="D37" s="6" t="n"/>
+      <c r="E37" s="8" t="n"/>
+      <c r="G37" s="5" t="n"/>
+      <c r="H37" s="6" t="n"/>
+      <c r="I37" s="7" t="n"/>
+      <c r="J37" s="6" t="n"/>
+      <c r="K37" s="8" t="n"/>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="9" t="n"/>
       <c r="B38" s="10" t="n"/>
       <c r="C38" s="11" t="n"/>
-      <c r="D38" s="12" t="n"/>
-      <c r="F38" s="9" t="n"/>
-      <c r="G38" s="10" t="n"/>
-      <c r="H38" s="11" t="n"/>
-      <c r="I38" s="12" t="n"/>
+      <c r="D38" s="10" t="n"/>
+      <c r="E38" s="12" t="n"/>
+      <c r="G38" s="9" t="n"/>
+      <c r="H38" s="10" t="n"/>
+      <c r="I38" s="11" t="n"/>
+      <c r="J38" s="10" t="n"/>
+      <c r="K38" s="12" t="n"/>
     </row>
     <row r="39" ht="15" customHeight="1">
       <c r="A39" s="9" t="n"/>
       <c r="B39" s="10" t="n"/>
       <c r="C39" s="11" t="n"/>
-      <c r="D39" s="12" t="n"/>
-      <c r="F39" s="9" t="n"/>
-      <c r="G39" s="10" t="n"/>
-      <c r="H39" s="11" t="n"/>
-      <c r="I39" s="12" t="n"/>
+      <c r="D39" s="10" t="n"/>
+      <c r="E39" s="12" t="n"/>
+      <c r="G39" s="9" t="n"/>
+      <c r="H39" s="10" t="n"/>
+      <c r="I39" s="11" t="n"/>
+      <c r="J39" s="10" t="n"/>
+      <c r="K39" s="12" t="n"/>
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="A40" s="13" t="n"/>
       <c r="B40" s="14" t="n"/>
       <c r="C40" s="15" t="n"/>
-      <c r="D40" s="16" t="n"/>
-      <c r="F40" s="13" t="n"/>
-      <c r="G40" s="14" t="n"/>
-      <c r="H40" s="15" t="n"/>
-      <c r="I40" s="16" t="n"/>
+      <c r="D40" s="14" t="n"/>
+      <c r="E40" s="16" t="n"/>
+      <c r="G40" s="13" t="n"/>
+      <c r="H40" s="14" t="n"/>
+      <c r="I40" s="15" t="n"/>
+      <c r="J40" s="14" t="n"/>
+      <c r="K40" s="16" t="n"/>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" s="17" t="n"/>
       <c r="B41" s="18" t="n"/>
       <c r="C41" s="19" t="n"/>
-      <c r="D41" s="20" t="n"/>
-      <c r="F41" s="17" t="n"/>
-      <c r="G41" s="18" t="n"/>
-      <c r="H41" s="19" t="n"/>
-      <c r="I41" s="20" t="n"/>
+      <c r="D41" s="18" t="n"/>
+      <c r="E41" s="20" t="n"/>
+      <c r="G41" s="17" t="n"/>
+      <c r="H41" s="18" t="n"/>
+      <c r="I41" s="19" t="n"/>
+      <c r="J41" s="18" t="n"/>
+      <c r="K41" s="20" t="n"/>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="21" t="n"/>
       <c r="B42" s="22" t="n"/>
       <c r="C42" s="23" t="n"/>
-      <c r="D42" s="24" t="n"/>
-      <c r="F42" s="21" t="n"/>
-      <c r="G42" s="22" t="n"/>
-      <c r="H42" s="23" t="n"/>
-      <c r="I42" s="24" t="n"/>
+      <c r="D42" s="22" t="n"/>
+      <c r="E42" s="24" t="n"/>
+      <c r="G42" s="21" t="n"/>
+      <c r="H42" s="22" t="n"/>
+      <c r="I42" s="23" t="n"/>
+      <c r="J42" s="22" t="n"/>
+      <c r="K42" s="24" t="n"/>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" s="21" t="n"/>
       <c r="B43" s="22" t="n"/>
       <c r="C43" s="23" t="n"/>
-      <c r="D43" s="24" t="n"/>
-      <c r="F43" s="21" t="n"/>
-      <c r="G43" s="22" t="n"/>
-      <c r="H43" s="23" t="n"/>
-      <c r="I43" s="24" t="n"/>
+      <c r="D43" s="22" t="n"/>
+      <c r="E43" s="24" t="n"/>
+      <c r="G43" s="21" t="n"/>
+      <c r="H43" s="22" t="n"/>
+      <c r="I43" s="23" t="n"/>
+      <c r="J43" s="22" t="n"/>
+      <c r="K43" s="24" t="n"/>
     </row>
     <row r="44" ht="15" customHeight="1">
       <c r="A44" s="25" t="n"/>
       <c r="B44" s="26" t="n"/>
       <c r="C44" s="27" t="n"/>
-      <c r="D44" s="28" t="n"/>
-      <c r="F44" s="25" t="n"/>
-      <c r="G44" s="26" t="n"/>
-      <c r="H44" s="27" t="n"/>
-      <c r="I44" s="28" t="n"/>
+      <c r="D44" s="26" t="n"/>
+      <c r="E44" s="28" t="n"/>
+      <c r="G44" s="25" t="n"/>
+      <c r="H44" s="26" t="n"/>
+      <c r="I44" s="27" t="n"/>
+      <c r="J44" s="26" t="n"/>
+      <c r="K44" s="28" t="n"/>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="5" t="n"/>
       <c r="B45" s="6" t="n"/>
       <c r="C45" s="7" t="n"/>
-      <c r="D45" s="8" t="n"/>
-      <c r="F45" s="5" t="n"/>
-      <c r="G45" s="6" t="n"/>
-      <c r="H45" s="7" t="n"/>
-      <c r="I45" s="8" t="n"/>
+      <c r="D45" s="6" t="n"/>
+      <c r="E45" s="8" t="n"/>
+      <c r="G45" s="5" t="n"/>
+      <c r="H45" s="6" t="n"/>
+      <c r="I45" s="7" t="n"/>
+      <c r="J45" s="6" t="n"/>
+      <c r="K45" s="8" t="n"/>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="9" t="n"/>
       <c r="B46" s="10" t="n"/>
       <c r="C46" s="11" t="n"/>
-      <c r="D46" s="12" t="n"/>
-      <c r="F46" s="9" t="n"/>
-      <c r="G46" s="10" t="n"/>
-      <c r="H46" s="11" t="n"/>
-      <c r="I46" s="12" t="n"/>
+      <c r="D46" s="10" t="n"/>
+      <c r="E46" s="12" t="n"/>
+      <c r="G46" s="9" t="n"/>
+      <c r="H46" s="10" t="n"/>
+      <c r="I46" s="11" t="n"/>
+      <c r="J46" s="10" t="n"/>
+      <c r="K46" s="12" t="n"/>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="9" t="n"/>
       <c r="B47" s="10" t="n"/>
       <c r="C47" s="11" t="n"/>
-      <c r="D47" s="12" t="n"/>
-      <c r="F47" s="9" t="n"/>
-      <c r="G47" s="10" t="n"/>
-      <c r="H47" s="11" t="n"/>
-      <c r="I47" s="12" t="n"/>
+      <c r="D47" s="10" t="n"/>
+      <c r="E47" s="12" t="n"/>
+      <c r="G47" s="9" t="n"/>
+      <c r="H47" s="10" t="n"/>
+      <c r="I47" s="11" t="n"/>
+      <c r="J47" s="10" t="n"/>
+      <c r="K47" s="12" t="n"/>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="13" t="n"/>
       <c r="B48" s="14" t="n"/>
       <c r="C48" s="15" t="n"/>
-      <c r="D48" s="16" t="n"/>
-      <c r="F48" s="13" t="n"/>
-      <c r="G48" s="14" t="n"/>
-      <c r="H48" s="15" t="n"/>
-      <c r="I48" s="16" t="n"/>
+      <c r="D48" s="14" t="n"/>
+      <c r="E48" s="16" t="n"/>
+      <c r="G48" s="13" t="n"/>
+      <c r="H48" s="14" t="n"/>
+      <c r="I48" s="15" t="n"/>
+      <c r="J48" s="14" t="n"/>
+      <c r="K48" s="16" t="n"/>
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="A49" s="17" t="n"/>
       <c r="B49" s="18" t="n"/>
       <c r="C49" s="19" t="n"/>
-      <c r="D49" s="20" t="n"/>
-      <c r="F49" s="17" t="n"/>
-      <c r="G49" s="18" t="n"/>
-      <c r="H49" s="19" t="n"/>
-      <c r="I49" s="20" t="n"/>
+      <c r="D49" s="18" t="n"/>
+      <c r="E49" s="20" t="n"/>
+      <c r="G49" s="17" t="n"/>
+      <c r="H49" s="18" t="n"/>
+      <c r="I49" s="19" t="n"/>
+      <c r="J49" s="18" t="n"/>
+      <c r="K49" s="20" t="n"/>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="21" t="n"/>
       <c r="B50" s="22" t="n"/>
       <c r="C50" s="23" t="n"/>
-      <c r="D50" s="24" t="n"/>
-      <c r="F50" s="21" t="n"/>
-      <c r="G50" s="22" t="n"/>
-      <c r="H50" s="23" t="n"/>
-      <c r="I50" s="24" t="n"/>
+      <c r="D50" s="22" t="n"/>
+      <c r="E50" s="24" t="n"/>
+      <c r="G50" s="21" t="n"/>
+      <c r="H50" s="22" t="n"/>
+      <c r="I50" s="23" t="n"/>
+      <c r="J50" s="22" t="n"/>
+      <c r="K50" s="24" t="n"/>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" s="21" t="n"/>
       <c r="B51" s="22" t="n"/>
       <c r="C51" s="23" t="n"/>
-      <c r="D51" s="24" t="n"/>
-      <c r="F51" s="21" t="n"/>
-      <c r="G51" s="22" t="n"/>
-      <c r="H51" s="23" t="n"/>
-      <c r="I51" s="24" t="n"/>
+      <c r="D51" s="22" t="n"/>
+      <c r="E51" s="24" t="n"/>
+      <c r="G51" s="21" t="n"/>
+      <c r="H51" s="22" t="n"/>
+      <c r="I51" s="23" t="n"/>
+      <c r="J51" s="22" t="n"/>
+      <c r="K51" s="24" t="n"/>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="A52" s="25" t="n"/>
       <c r="B52" s="26" t="n"/>
       <c r="C52" s="27" t="n"/>
-      <c r="D52" s="28" t="n"/>
-      <c r="F52" s="25" t="n"/>
-      <c r="G52" s="26" t="n"/>
-      <c r="H52" s="27" t="n"/>
-      <c r="I52" s="28" t="n"/>
+      <c r="D52" s="26" t="n"/>
+      <c r="E52" s="28" t="n"/>
+      <c r="G52" s="25" t="n"/>
+      <c r="H52" s="26" t="n"/>
+      <c r="I52" s="27" t="n"/>
+      <c r="J52" s="26" t="n"/>
+      <c r="K52" s="28" t="n"/>
     </row>
     <row r="53" ht="15" customHeight="1">
       <c r="A53" s="5" t="n"/>
       <c r="B53" s="6" t="n"/>
       <c r="C53" s="7" t="n"/>
-      <c r="D53" s="8" t="n"/>
-      <c r="F53" s="5" t="n"/>
-      <c r="G53" s="6" t="n"/>
-      <c r="H53" s="7" t="n"/>
-      <c r="I53" s="8" t="n"/>
+      <c r="D53" s="6" t="n"/>
+      <c r="E53" s="8" t="n"/>
+      <c r="G53" s="5" t="n"/>
+      <c r="H53" s="6" t="n"/>
+      <c r="I53" s="7" t="n"/>
+      <c r="J53" s="6" t="n"/>
+      <c r="K53" s="8" t="n"/>
     </row>
     <row r="54" ht="15" customHeight="1">
       <c r="A54" s="9" t="n"/>
       <c r="B54" s="10" t="n"/>
       <c r="C54" s="11" t="n"/>
-      <c r="D54" s="12" t="n"/>
-      <c r="F54" s="9" t="n"/>
-      <c r="G54" s="10" t="n"/>
-      <c r="H54" s="11" t="n"/>
-      <c r="I54" s="12" t="n"/>
+      <c r="D54" s="10" t="n"/>
+      <c r="E54" s="12" t="n"/>
+      <c r="G54" s="9" t="n"/>
+      <c r="H54" s="10" t="n"/>
+      <c r="I54" s="11" t="n"/>
+      <c r="J54" s="10" t="n"/>
+      <c r="K54" s="12" t="n"/>
     </row>
     <row r="55" ht="15" customHeight="1">
       <c r="A55" s="9" t="n"/>
       <c r="B55" s="10" t="n"/>
       <c r="C55" s="11" t="n"/>
-      <c r="D55" s="12" t="n"/>
-      <c r="F55" s="9" t="n"/>
-      <c r="G55" s="10" t="n"/>
-      <c r="H55" s="11" t="n"/>
-      <c r="I55" s="12" t="n"/>
+      <c r="D55" s="10" t="n"/>
+      <c r="E55" s="12" t="n"/>
+      <c r="G55" s="9" t="n"/>
+      <c r="H55" s="10" t="n"/>
+      <c r="I55" s="11" t="n"/>
+      <c r="J55" s="10" t="n"/>
+      <c r="K55" s="12" t="n"/>
     </row>
     <row r="56" ht="15" customHeight="1">
       <c r="A56" s="13" t="n"/>
       <c r="B56" s="14" t="n"/>
       <c r="C56" s="15" t="n"/>
-      <c r="D56" s="16" t="n"/>
-      <c r="F56" s="13" t="n"/>
-      <c r="G56" s="14" t="n"/>
-      <c r="H56" s="15" t="n"/>
-      <c r="I56" s="16" t="n"/>
+      <c r="D56" s="14" t="n"/>
+      <c r="E56" s="16" t="n"/>
+      <c r="G56" s="13" t="n"/>
+      <c r="H56" s="14" t="n"/>
+      <c r="I56" s="15" t="n"/>
+      <c r="J56" s="14" t="n"/>
+      <c r="K56" s="16" t="n"/>
     </row>
     <row r="57" ht="15" customHeight="1">
       <c r="A57" s="17" t="n"/>
       <c r="B57" s="18" t="n"/>
       <c r="C57" s="19" t="n"/>
-      <c r="D57" s="20" t="n"/>
-      <c r="F57" s="17" t="n"/>
-      <c r="G57" s="18" t="n"/>
-      <c r="H57" s="19" t="n"/>
-      <c r="I57" s="20" t="n"/>
+      <c r="D57" s="18" t="n"/>
+      <c r="E57" s="20" t="n"/>
+      <c r="G57" s="17" t="n"/>
+      <c r="H57" s="18" t="n"/>
+      <c r="I57" s="19" t="n"/>
+      <c r="J57" s="18" t="n"/>
+      <c r="K57" s="20" t="n"/>
     </row>
     <row r="58" ht="15" customHeight="1">
       <c r="A58" s="21" t="n"/>
       <c r="B58" s="22" t="n"/>
       <c r="C58" s="23" t="n"/>
-      <c r="D58" s="24" t="n"/>
-      <c r="F58" s="21" t="n"/>
-      <c r="G58" s="22" t="n"/>
-      <c r="H58" s="23" t="n"/>
-      <c r="I58" s="24" t="n"/>
+      <c r="D58" s="22" t="n"/>
+      <c r="E58" s="24" t="n"/>
+      <c r="G58" s="21" t="n"/>
+      <c r="H58" s="22" t="n"/>
+      <c r="I58" s="23" t="n"/>
+      <c r="J58" s="22" t="n"/>
+      <c r="K58" s="24" t="n"/>
     </row>
     <row r="59" ht="15" customHeight="1">
       <c r="A59" s="21" t="n"/>
       <c r="B59" s="22" t="n"/>
       <c r="C59" s="23" t="n"/>
-      <c r="D59" s="24" t="n"/>
-      <c r="F59" s="21" t="n"/>
-      <c r="G59" s="22" t="n"/>
-      <c r="H59" s="23" t="n"/>
-      <c r="I59" s="24" t="n"/>
+      <c r="D59" s="22" t="n"/>
+      <c r="E59" s="24" t="n"/>
+      <c r="G59" s="21" t="n"/>
+      <c r="H59" s="22" t="n"/>
+      <c r="I59" s="23" t="n"/>
+      <c r="J59" s="22" t="n"/>
+      <c r="K59" s="24" t="n"/>
     </row>
     <row r="60" ht="15" customHeight="1">
       <c r="A60" s="25" t="n"/>
       <c r="B60" s="26" t="n"/>
       <c r="C60" s="27" t="n"/>
-      <c r="D60" s="28" t="n"/>
-      <c r="F60" s="25" t="n"/>
-      <c r="G60" s="26" t="n"/>
-      <c r="H60" s="27" t="n"/>
-      <c r="I60" s="28" t="n"/>
+      <c r="D60" s="26" t="n"/>
+      <c r="E60" s="28" t="n"/>
+      <c r="G60" s="25" t="n"/>
+      <c r="H60" s="26" t="n"/>
+      <c r="I60" s="27" t="n"/>
+      <c r="J60" s="26" t="n"/>
+      <c r="K60" s="28" t="n"/>
     </row>
     <row r="61" ht="15" customHeight="1">
       <c r="A61" s="5" t="n"/>
       <c r="B61" s="6" t="n"/>
       <c r="C61" s="7" t="n"/>
-      <c r="D61" s="8" t="n"/>
-      <c r="F61" s="5" t="n"/>
-      <c r="G61" s="6" t="n"/>
-      <c r="H61" s="7" t="n"/>
-      <c r="I61" s="8" t="n"/>
+      <c r="D61" s="6" t="n"/>
+      <c r="E61" s="8" t="n"/>
+      <c r="G61" s="5" t="n"/>
+      <c r="H61" s="6" t="n"/>
+      <c r="I61" s="7" t="n"/>
+      <c r="J61" s="6" t="n"/>
+      <c r="K61" s="8" t="n"/>
     </row>
     <row r="62" ht="15" customHeight="1">
       <c r="A62" s="9" t="n"/>
       <c r="B62" s="10" t="n"/>
       <c r="C62" s="11" t="n"/>
-      <c r="D62" s="12" t="n"/>
-      <c r="F62" s="9" t="n"/>
-      <c r="G62" s="10" t="n"/>
-      <c r="H62" s="11" t="n"/>
-      <c r="I62" s="12" t="n"/>
+      <c r="D62" s="10" t="n"/>
+      <c r="E62" s="12" t="n"/>
+      <c r="G62" s="9" t="n"/>
+      <c r="H62" s="10" t="n"/>
+      <c r="I62" s="11" t="n"/>
+      <c r="J62" s="10" t="n"/>
+      <c r="K62" s="12" t="n"/>
     </row>
     <row r="63" ht="15" customHeight="1">
       <c r="A63" s="9" t="n"/>
       <c r="B63" s="10" t="n"/>
       <c r="C63" s="11" t="n"/>
-      <c r="D63" s="12" t="n"/>
-      <c r="F63" s="9" t="n"/>
-      <c r="G63" s="10" t="n"/>
-      <c r="H63" s="11" t="n"/>
-      <c r="I63" s="12" t="n"/>
+      <c r="D63" s="10" t="n"/>
+      <c r="E63" s="12" t="n"/>
+      <c r="G63" s="9" t="n"/>
+      <c r="H63" s="10" t="n"/>
+      <c r="I63" s="11" t="n"/>
+      <c r="J63" s="10" t="n"/>
+      <c r="K63" s="12" t="n"/>
     </row>
     <row r="64" ht="15" customHeight="1">
       <c r="A64" s="13" t="n"/>
       <c r="B64" s="14" t="n"/>
       <c r="C64" s="15" t="n"/>
-      <c r="D64" s="16" t="n"/>
-      <c r="F64" s="13" t="n"/>
-      <c r="G64" s="14" t="n"/>
-      <c r="H64" s="15" t="n"/>
-      <c r="I64" s="16" t="n"/>
+      <c r="D64" s="14" t="n"/>
+      <c r="E64" s="16" t="n"/>
+      <c r="G64" s="13" t="n"/>
+      <c r="H64" s="14" t="n"/>
+      <c r="I64" s="15" t="n"/>
+      <c r="J64" s="14" t="n"/>
+      <c r="K64" s="16" t="n"/>
     </row>
     <row r="65" ht="15" customHeight="1">
       <c r="A65" s="17" t="n"/>
       <c r="B65" s="18" t="n"/>
       <c r="C65" s="19" t="n"/>
-      <c r="D65" s="20" t="n"/>
-      <c r="F65" s="17" t="n"/>
-      <c r="G65" s="18" t="n"/>
-      <c r="H65" s="19" t="n"/>
-      <c r="I65" s="20" t="n"/>
+      <c r="D65" s="18" t="n"/>
+      <c r="E65" s="20" t="n"/>
+      <c r="G65" s="17" t="n"/>
+      <c r="H65" s="18" t="n"/>
+      <c r="I65" s="19" t="n"/>
+      <c r="J65" s="18" t="n"/>
+      <c r="K65" s="20" t="n"/>
     </row>
     <row r="66" ht="15" customHeight="1">
       <c r="A66" s="21" t="n"/>
       <c r="B66" s="22" t="n"/>
       <c r="C66" s="23" t="n"/>
-      <c r="D66" s="24" t="n"/>
-      <c r="F66" s="21" t="n"/>
-      <c r="G66" s="22" t="n"/>
-      <c r="H66" s="23" t="n"/>
-      <c r="I66" s="24" t="n"/>
+      <c r="D66" s="22" t="n"/>
+      <c r="E66" s="24" t="n"/>
+      <c r="G66" s="21" t="n"/>
+      <c r="H66" s="22" t="n"/>
+      <c r="I66" s="23" t="n"/>
+      <c r="J66" s="22" t="n"/>
+      <c r="K66" s="24" t="n"/>
     </row>
     <row r="67" ht="15" customHeight="1">
       <c r="A67" s="21" t="n"/>
       <c r="B67" s="22" t="n"/>
       <c r="C67" s="23" t="n"/>
-      <c r="D67" s="24" t="n"/>
-      <c r="F67" s="21" t="n"/>
-      <c r="G67" s="22" t="n"/>
-      <c r="H67" s="23" t="n"/>
-      <c r="I67" s="24" t="n"/>
+      <c r="D67" s="22" t="n"/>
+      <c r="E67" s="24" t="n"/>
+      <c r="G67" s="21" t="n"/>
+      <c r="H67" s="22" t="n"/>
+      <c r="I67" s="23" t="n"/>
+      <c r="J67" s="22" t="n"/>
+      <c r="K67" s="24" t="n"/>
     </row>
     <row r="68" ht="15" customHeight="1">
       <c r="A68" s="25" t="n"/>
       <c r="B68" s="26" t="n"/>
       <c r="C68" s="27" t="n"/>
-      <c r="D68" s="28" t="n"/>
-      <c r="F68" s="25" t="n"/>
-      <c r="G68" s="26" t="n"/>
-      <c r="H68" s="27" t="n"/>
-      <c r="I68" s="28" t="n"/>
+      <c r="D68" s="26" t="n"/>
+      <c r="E68" s="28" t="n"/>
+      <c r="G68" s="25" t="n"/>
+      <c r="H68" s="26" t="n"/>
+      <c r="I68" s="27" t="n"/>
+      <c r="J68" s="26" t="n"/>
+      <c r="K68" s="28" t="n"/>
     </row>
     <row r="69" ht="15" customHeight="1">
       <c r="A69" s="5" t="n"/>
       <c r="B69" s="6" t="n"/>
       <c r="C69" s="7" t="n"/>
-      <c r="D69" s="8" t="n"/>
-      <c r="F69" s="5" t="n"/>
-      <c r="G69" s="6" t="n"/>
-      <c r="H69" s="7" t="n"/>
-      <c r="I69" s="8" t="n"/>
+      <c r="D69" s="6" t="n"/>
+      <c r="E69" s="8" t="n"/>
+      <c r="G69" s="5" t="n"/>
+      <c r="H69" s="6" t="n"/>
+      <c r="I69" s="7" t="n"/>
+      <c r="J69" s="6" t="n"/>
+      <c r="K69" s="8" t="n"/>
     </row>
     <row r="70" ht="15" customHeight="1">
       <c r="A70" s="9" t="n"/>
       <c r="B70" s="10" t="n"/>
       <c r="C70" s="11" t="n"/>
-      <c r="D70" s="12" t="n"/>
-      <c r="F70" s="9" t="n"/>
-      <c r="G70" s="10" t="n"/>
-      <c r="H70" s="11" t="n"/>
-      <c r="I70" s="12" t="n"/>
+      <c r="D70" s="10" t="n"/>
+      <c r="E70" s="12" t="n"/>
+      <c r="G70" s="9" t="n"/>
+      <c r="H70" s="10" t="n"/>
+      <c r="I70" s="11" t="n"/>
+      <c r="J70" s="10" t="n"/>
+      <c r="K70" s="12" t="n"/>
     </row>
     <row r="71" ht="15" customHeight="1">
       <c r="A71" s="9" t="n"/>
       <c r="B71" s="10" t="n"/>
       <c r="C71" s="11" t="n"/>
-      <c r="D71" s="12" t="n"/>
-      <c r="F71" s="9" t="n"/>
-      <c r="G71" s="10" t="n"/>
-      <c r="H71" s="11" t="n"/>
-      <c r="I71" s="12" t="n"/>
+      <c r="D71" s="10" t="n"/>
+      <c r="E71" s="12" t="n"/>
+      <c r="G71" s="9" t="n"/>
+      <c r="H71" s="10" t="n"/>
+      <c r="I71" s="11" t="n"/>
+      <c r="J71" s="10" t="n"/>
+      <c r="K71" s="12" t="n"/>
     </row>
     <row r="72" ht="15" customHeight="1">
       <c r="A72" s="13" t="n"/>
       <c r="B72" s="14" t="n"/>
       <c r="C72" s="15" t="n"/>
-      <c r="D72" s="16" t="n"/>
-      <c r="F72" s="13" t="n"/>
-      <c r="G72" s="14" t="n"/>
-      <c r="H72" s="15" t="n"/>
-      <c r="I72" s="16" t="n"/>
+      <c r="D72" s="14" t="n"/>
+      <c r="E72" s="16" t="n"/>
+      <c r="G72" s="13" t="n"/>
+      <c r="H72" s="14" t="n"/>
+      <c r="I72" s="15" t="n"/>
+      <c r="J72" s="14" t="n"/>
+      <c r="K72" s="16" t="n"/>
     </row>
     <row r="73" ht="15" customHeight="1">
       <c r="A73" s="17" t="n"/>
       <c r="B73" s="18" t="n"/>
       <c r="C73" s="19" t="n"/>
-      <c r="D73" s="20" t="n"/>
-      <c r="F73" s="17" t="n"/>
-      <c r="G73" s="18" t="n"/>
-      <c r="H73" s="19" t="n"/>
-      <c r="I73" s="20" t="n"/>
+      <c r="D73" s="18" t="n"/>
+      <c r="E73" s="20" t="n"/>
+      <c r="G73" s="17" t="n"/>
+      <c r="H73" s="18" t="n"/>
+      <c r="I73" s="19" t="n"/>
+      <c r="J73" s="18" t="n"/>
+      <c r="K73" s="20" t="n"/>
     </row>
     <row r="74" ht="15" customHeight="1">
       <c r="A74" s="21" t="n"/>
       <c r="B74" s="22" t="n"/>
       <c r="C74" s="23" t="n"/>
-      <c r="D74" s="24" t="n"/>
-      <c r="F74" s="21" t="n"/>
-      <c r="G74" s="22" t="n"/>
-      <c r="H74" s="23" t="n"/>
-      <c r="I74" s="24" t="n"/>
+      <c r="D74" s="22" t="n"/>
+      <c r="E74" s="24" t="n"/>
+      <c r="G74" s="21" t="n"/>
+      <c r="H74" s="22" t="n"/>
+      <c r="I74" s="23" t="n"/>
+      <c r="J74" s="22" t="n"/>
+      <c r="K74" s="24" t="n"/>
     </row>
     <row r="75" ht="15" customHeight="1">
       <c r="A75" s="21" t="n"/>
       <c r="B75" s="22" t="n"/>
       <c r="C75" s="23" t="n"/>
-      <c r="D75" s="24" t="n"/>
-      <c r="F75" s="21" t="n"/>
-      <c r="G75" s="22" t="n"/>
-      <c r="H75" s="23" t="n"/>
-      <c r="I75" s="24" t="n"/>
+      <c r="D75" s="22" t="n"/>
+      <c r="E75" s="24" t="n"/>
+      <c r="G75" s="21" t="n"/>
+      <c r="H75" s="22" t="n"/>
+      <c r="I75" s="23" t="n"/>
+      <c r="J75" s="22" t="n"/>
+      <c r="K75" s="24" t="n"/>
     </row>
     <row r="76" ht="15" customHeight="1">
       <c r="A76" s="25" t="n"/>
       <c r="B76" s="26" t="n"/>
       <c r="C76" s="27" t="n"/>
-      <c r="D76" s="28" t="n"/>
-      <c r="F76" s="25" t="n"/>
-      <c r="G76" s="26" t="n"/>
-      <c r="H76" s="27" t="n"/>
-      <c r="I76" s="28" t="n"/>
+      <c r="D76" s="26" t="n"/>
+      <c r="E76" s="28" t="n"/>
+      <c r="G76" s="25" t="n"/>
+      <c r="H76" s="26" t="n"/>
+      <c r="I76" s="27" t="n"/>
+      <c r="J76" s="26" t="n"/>
+      <c r="K76" s="28" t="n"/>
     </row>
     <row r="77" ht="15" customHeight="1">
       <c r="A77" s="5" t="n"/>
       <c r="B77" s="6" t="n"/>
       <c r="C77" s="7" t="n"/>
-      <c r="D77" s="8" t="n"/>
-      <c r="F77" s="5" t="n"/>
-      <c r="G77" s="6" t="n"/>
-      <c r="H77" s="7" t="n"/>
-      <c r="I77" s="8" t="n"/>
+      <c r="D77" s="6" t="n"/>
+      <c r="E77" s="8" t="n"/>
+      <c r="G77" s="5" t="n"/>
+      <c r="H77" s="6" t="n"/>
+      <c r="I77" s="7" t="n"/>
+      <c r="J77" s="6" t="n"/>
+      <c r="K77" s="8" t="n"/>
     </row>
     <row r="78" ht="15" customHeight="1">
       <c r="A78" s="9" t="n"/>
       <c r="B78" s="10" t="n"/>
       <c r="C78" s="11" t="n"/>
-      <c r="D78" s="12" t="n"/>
-      <c r="F78" s="9" t="n"/>
-      <c r="G78" s="10" t="n"/>
-      <c r="H78" s="11" t="n"/>
-      <c r="I78" s="12" t="n"/>
+      <c r="D78" s="10" t="n"/>
+      <c r="E78" s="12" t="n"/>
+      <c r="G78" s="9" t="n"/>
+      <c r="H78" s="10" t="n"/>
+      <c r="I78" s="11" t="n"/>
+      <c r="J78" s="10" t="n"/>
+      <c r="K78" s="12" t="n"/>
     </row>
     <row r="79" ht="15" customHeight="1">
       <c r="A79" s="9" t="n"/>
       <c r="B79" s="10" t="n"/>
       <c r="C79" s="11" t="n"/>
-      <c r="D79" s="12" t="n"/>
-      <c r="F79" s="9" t="n"/>
-      <c r="G79" s="10" t="n"/>
-      <c r="H79" s="11" t="n"/>
-      <c r="I79" s="12" t="n"/>
+      <c r="D79" s="10" t="n"/>
+      <c r="E79" s="12" t="n"/>
+      <c r="G79" s="9" t="n"/>
+      <c r="H79" s="10" t="n"/>
+      <c r="I79" s="11" t="n"/>
+      <c r="J79" s="10" t="n"/>
+      <c r="K79" s="12" t="n"/>
     </row>
     <row r="80" ht="15" customHeight="1">
       <c r="A80" s="13" t="n"/>
       <c r="B80" s="14" t="n"/>
       <c r="C80" s="15" t="n"/>
-      <c r="D80" s="16" t="n"/>
-      <c r="F80" s="13" t="n"/>
-      <c r="G80" s="14" t="n"/>
-      <c r="H80" s="15" t="n"/>
-      <c r="I80" s="16" t="n"/>
+      <c r="D80" s="14" t="n"/>
+      <c r="E80" s="16" t="n"/>
+      <c r="G80" s="13" t="n"/>
+      <c r="H80" s="14" t="n"/>
+      <c r="I80" s="15" t="n"/>
+      <c r="J80" s="14" t="n"/>
+      <c r="K80" s="16" t="n"/>
     </row>
     <row r="81" ht="15" customHeight="1">
       <c r="A81" s="17" t="n"/>
       <c r="B81" s="18" t="n"/>
       <c r="C81" s="19" t="n"/>
-      <c r="D81" s="20" t="n"/>
-      <c r="F81" s="17" t="n"/>
-      <c r="G81" s="18" t="n"/>
-      <c r="H81" s="19" t="n"/>
-      <c r="I81" s="20" t="n"/>
+      <c r="D81" s="18" t="n"/>
+      <c r="E81" s="20" t="n"/>
+      <c r="G81" s="17" t="n"/>
+      <c r="H81" s="18" t="n"/>
+      <c r="I81" s="19" t="n"/>
+      <c r="J81" s="18" t="n"/>
+      <c r="K81" s="20" t="n"/>
     </row>
     <row r="82" ht="15" customHeight="1">
       <c r="A82" s="21" t="n"/>
       <c r="B82" s="22" t="n"/>
       <c r="C82" s="23" t="n"/>
-      <c r="D82" s="24" t="n"/>
-      <c r="F82" s="21" t="n"/>
-      <c r="G82" s="22" t="n"/>
-      <c r="H82" s="23" t="n"/>
-      <c r="I82" s="24" t="n"/>
+      <c r="D82" s="22" t="n"/>
+      <c r="E82" s="24" t="n"/>
+      <c r="G82" s="21" t="n"/>
+      <c r="H82" s="22" t="n"/>
+      <c r="I82" s="23" t="n"/>
+      <c r="J82" s="22" t="n"/>
+      <c r="K82" s="24" t="n"/>
     </row>
     <row r="83" ht="15" customHeight="1">
       <c r="A83" s="21" t="n"/>
       <c r="B83" s="22" t="n"/>
       <c r="C83" s="23" t="n"/>
-      <c r="D83" s="24" t="n"/>
-      <c r="F83" s="21" t="n"/>
-      <c r="G83" s="22" t="n"/>
-      <c r="H83" s="23" t="n"/>
-      <c r="I83" s="24" t="n"/>
+      <c r="D83" s="22" t="n"/>
+      <c r="E83" s="24" t="n"/>
+      <c r="G83" s="21" t="n"/>
+      <c r="H83" s="22" t="n"/>
+      <c r="I83" s="23" t="n"/>
+      <c r="J83" s="22" t="n"/>
+      <c r="K83" s="24" t="n"/>
     </row>
     <row r="84" ht="15" customHeight="1">
       <c r="A84" s="25" t="n"/>
       <c r="B84" s="26" t="n"/>
       <c r="C84" s="27" t="n"/>
-      <c r="D84" s="28" t="n"/>
-      <c r="F84" s="25" t="n"/>
-      <c r="G84" s="26" t="n"/>
-      <c r="H84" s="27" t="n"/>
-      <c r="I84" s="28" t="n"/>
+      <c r="D84" s="26" t="n"/>
+      <c r="E84" s="28" t="n"/>
+      <c r="G84" s="25" t="n"/>
+      <c r="H84" s="26" t="n"/>
+      <c r="I84" s="27" t="n"/>
+      <c r="J84" s="26" t="n"/>
+      <c r="K84" s="28" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.6" header="0.3" footer="0.3"/>

</xml_diff>